<commit_message>
Rework retry/error handling, fix Excel output, refresh demo data
- Retry only on network errors, 5xx and 429; 4xx fails fast without retries
- Track incomplete categories (missing pages, empty pages, card parse
  errors) instead of a flat error counter; exit with code 1 when any
  category is incomplete
- Save price as a numeric column with currency format instead of text,
  add clickable hyperlinks, autofilter and a frozen header row
- Point the User-Agent at the GitHub repo instead of a placeholder URL
- Regenerate output/books.xlsx, output/travel.xlsx and the README
  screenshot from the updated script so the portfolio demo matches
  what the code actually produces

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/travel.xlsx
+++ b/output/travel.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$F$12</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,6 +29,13 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,17 +61,21 @@
       <bottom style="thin"/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -429,7 +442,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
@@ -444,7 +457,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Цена</t>
+          <t>Цена, £</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -474,10 +487,8 @@
           <t>It's Only the Himalayas</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>£45.17</t>
-        </is>
+      <c r="B2" s="2" t="n">
+        <v>45.17</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -492,7 +503,7 @@
       <c r="E2" t="n">
         <v>2</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>http://books.toscrape.com/catalogue/its-only-the-himalayas_981/index.html</t>
         </is>
@@ -504,10 +515,8 @@
           <t>Full Moon over Noah’s Ark: An Odyssey to Mount Ararat and Beyond</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>£49.43</t>
-        </is>
+      <c r="B3" s="2" t="n">
+        <v>49.43</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -522,7 +531,7 @@
       <c r="E3" t="n">
         <v>4</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>http://books.toscrape.com/catalogue/full-moon-over-noahs-ark-an-odyssey-to-mount-ararat-and-beyond_811/index.html</t>
         </is>
@@ -534,10 +543,8 @@
           <t>See America: A Celebration of Our National Parks &amp; Treasured Sites</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>£48.87</t>
-        </is>
+      <c r="B4" s="2" t="n">
+        <v>48.87</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -552,7 +559,7 @@
       <c r="E4" t="n">
         <v>3</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>http://books.toscrape.com/catalogue/see-america-a-celebration-of-our-national-parks-treasured-sites_732/index.html</t>
         </is>
@@ -564,10 +571,8 @@
           <t>Vagabonding: An Uncommon Guide to the Art of Long-Term World Travel</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>£36.94</t>
-        </is>
+      <c r="B5" s="2" t="n">
+        <v>36.94</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -582,7 +587,7 @@
       <c r="E5" t="n">
         <v>2</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>http://books.toscrape.com/catalogue/vagabonding-an-uncommon-guide-to-the-art-of-long-term-world-travel_552/index.html</t>
         </is>
@@ -594,10 +599,8 @@
           <t>Under the Tuscan Sun</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>£37.33</t>
-        </is>
+      <c r="B6" s="2" t="n">
+        <v>37.33</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -612,7 +615,7 @@
       <c r="E6" t="n">
         <v>3</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>http://books.toscrape.com/catalogue/under-the-tuscan-sun_504/index.html</t>
         </is>
@@ -624,10 +627,8 @@
           <t>A Summer In Europe</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>£44.34</t>
-        </is>
+      <c r="B7" s="2" t="n">
+        <v>44.34</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -642,7 +643,7 @@
       <c r="E7" t="n">
         <v>2</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>http://books.toscrape.com/catalogue/a-summer-in-europe_458/index.html</t>
         </is>
@@ -654,10 +655,8 @@
           <t>The Great Railway Bazaar</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>£30.54</t>
-        </is>
+      <c r="B8" s="2" t="n">
+        <v>30.54</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -672,7 +671,7 @@
       <c r="E8" t="n">
         <v>1</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>http://books.toscrape.com/catalogue/the-great-railway-bazaar_446/index.html</t>
         </is>
@@ -684,10 +683,8 @@
           <t>A Year in Provence (Provence #1)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>£56.88</t>
-        </is>
+      <c r="B9" s="2" t="n">
+        <v>56.88</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -702,7 +699,7 @@
       <c r="E9" t="n">
         <v>4</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>http://books.toscrape.com/catalogue/a-year-in-provence-provence-1_421/index.html</t>
         </is>
@@ -714,10 +711,8 @@
           <t>The Road to Little Dribbling: Adventures of an American in Britain (Notes From a Small Island #2)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>£23.21</t>
-        </is>
+      <c r="B10" s="2" t="n">
+        <v>23.21</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -732,7 +727,7 @@
       <c r="E10" t="n">
         <v>1</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>http://books.toscrape.com/catalogue/the-road-to-little-dribbling-adventures-of-an-american-in-britain-notes-from-a-small-island-2_277/index.html</t>
         </is>
@@ -744,10 +739,8 @@
           <t>Neither Here nor There: Travels in Europe</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>£38.95</t>
-        </is>
+      <c r="B11" s="2" t="n">
+        <v>38.95</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -762,7 +755,7 @@
       <c r="E11" t="n">
         <v>3</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>http://books.toscrape.com/catalogue/neither-here-nor-there-travels-in-europe_198/index.html</t>
         </is>
@@ -774,10 +767,8 @@
           <t>1,000 Places to See Before You Die</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>£26.08</t>
-        </is>
+      <c r="B12" s="2" t="n">
+        <v>26.08</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -792,13 +783,27 @@
       <c r="E12" t="n">
         <v>5</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>http://books.toscrape.com/catalogue/1000-places-to-see-before-you-die_1/index.html</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F12"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId11"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>